<commit_message>
Studio 9: two parts, Smartsheet then Colab, on one conference workbook
Part 1 imports the conference workbook into Smartsheet, turns on
dependencies, shows the critical path, uses per-person filters to see
who is double-booked, and resolves one conflict with a resource link.
Part 2 runs the levelling notebook at two and three coordinators and
prices the heuristic against the optimum. Hand levelling, the budget,
the loan scenario and the AI reconciliation are removed from the studio.

The workbook is now a single clean worksheet with Start and End Date
columns; the note row that would have imported as a stray row and the
Formulas tab are gone. The notebook downloads the same workbook by
default, with upload and inline-table options. The week page's
Smartsheet steps and the deck's studio slides follow the new layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/week-09-smartsheet-resource-workout.xlsx
+++ b/files/week-09-smartsheet-resource-workout.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Smartsheet Import" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,10 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +32,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="3">
@@ -76,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,12 +84,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,17 +455,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -495,22 +492,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Allocation %</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Coordinators</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Cost</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Coordinators needed</t>
         </is>
       </c>
     </row>
@@ -531,20 +533,21 @@
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>2000</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I2" s="5" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -567,20 +570,19 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Kim, Lee</t>
         </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>30000</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I3" s="5" t="n">
+        <v>30000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -603,20 +605,19 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Ortiz</t>
         </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>6000</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I4" s="5" t="n">
+        <v>6000</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -639,20 +640,19 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>8000</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I5" s="5" t="n">
+        <v>8000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -675,20 +675,19 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Lee, Ortiz</t>
         </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>12000</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I6" s="5" t="n">
+        <v>12000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -711,20 +710,19 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Kim, Lee</t>
         </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>2500</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I7" s="5" t="n">
+        <v>2500</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -747,20 +745,19 @@
           <t>4, 5</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>3000</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I8" s="5" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -783,20 +780,19 @@
           <t>6, 7</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Kim, Lee</t>
         </is>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>4000</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I9" s="5" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -819,411 +815,18 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Lee, Ortiz</t>
         </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>2500</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Import this tab. Predecessors are Smartsheet row numbers (A = row 1). Assigned To holds the early-start assignment of three coordinators; Allocation % is 100 per person.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Column or field</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Smartsheet formula</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Cost per day</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C2" s="6">
-        <f>Cost@row / NETWORKDAYS([Start Date]@row, [End Date]@row)</f>
-        <v/>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Direct cost spread evenly over the activity's workdays</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Workday start</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C3" s="6">
-        <f>NETWORKDAYS([Start Date]$1, [Start Date]@row) - 1</f>
-        <v/>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>0 = project start; matches the notes' day numbers</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Workday finish</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C4" s="6">
-        <f>NETWORKDAYS([Start Date]$1, [End Date]@row)</f>
-        <v/>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Finish day as the notes count it</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Wk 1 PV</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C5" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 2), [Start Date]@row, DATE(2026, 11, 2)), IF([End Date]@row &lt; DATE(2026, 11, 6), [End Date]@row, DATE(2026, 11, 6)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 1: Mon 2 Nov to Fri 6 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Wk 2 PV</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C6" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 9), [Start Date]@row, DATE(2026, 11, 9)), IF([End Date]@row &lt; DATE(2026, 11, 13), [End Date]@row, DATE(2026, 11, 13)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 2: Mon 9 Nov to Fri 13 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Wk 3 PV</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C7" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 16), [Start Date]@row, DATE(2026, 11, 16)), IF([End Date]@row &lt; DATE(2026, 11, 20), [End Date]@row, DATE(2026, 11, 20)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 3: Mon 16 Nov to Fri 20 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Wk 4 PV</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C8" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 23), [Start Date]@row, DATE(2026, 11, 23)), IF([End Date]@row &lt; DATE(2026, 11, 27), [End Date]@row, DATE(2026, 11, 27)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 4: Mon 23 Nov to Fri 27 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Wk 5 PV</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C9" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 30), [Start Date]@row, DATE(2026, 11, 30)), IF([End Date]@row &lt; DATE(2026, 12, 4), [End Date]@row, DATE(2026, 12, 4)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 5: Mon 30 Nov to Fri 4 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Wk 6 PV</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C10" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 12, 7), [Start Date]@row, DATE(2026, 12, 7)), IF([End Date]@row &lt; DATE(2026, 12, 11), [End Date]@row, DATE(2026, 12, 11)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 6: Mon 7 Dec to Fri 11 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Wk 7 PV</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C11" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 12, 14), [Start Date]@row, DATE(2026, 12, 14)), IF([End Date]@row &lt; DATE(2026, 12, 18), [End Date]@row, DATE(2026, 12, 18)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 7: Mon 14 Dec to Fri 18 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Wk 8 PV</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C12" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 12, 21), [Start Date]@row, DATE(2026, 12, 21)), IF([End Date]@row &lt; DATE(2026, 12, 25), [End Date]@row, DATE(2026, 12, 25)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 8: Mon 21 Dec to Fri 25 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Project finish</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C13" s="6">
-        <f>MAX([End Date]:[End Date])</f>
-        <v/>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Date type</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Workdays</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C14" s="6">
-        <f>MAX([Workday finish]:[Workday finish])</f>
-        <v/>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>25 on the early-start schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Wk n total</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C15" s="6">
-        <f>SUM([Wk 1 PV]:[Wk 1 PV])  (one field per week)</f>
-        <v/>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Weekly planned value</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Cumulative to wk n</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C16" s="6">
-        <f>[Wk 1 total]# + [Wk 2 total]#  (extend per week)</f>
-        <v/>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>The baseline curve</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Total cost</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C17" s="6">
-        <f>SUM(Cost:Cost)</f>
-        <v/>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Must read $70,000 under every schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Smartsheet imports values, not formulas. Type each formula once in row 1, then right-click → Convert to Column Formula. Summary fields are typed in the Sheet Summary panel.</t>
-        </is>
+      <c r="I10" s="5" t="n">
+        <v>2500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish site (gated as of build date) 37ab8d664fa998eff7f12a4e8245b32b299de483
</commit_message>
<xml_diff>
--- a/files/week-09-smartsheet-resource-workout.xlsx
+++ b/files/week-09-smartsheet-resource-workout.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Smartsheet Import" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formulas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conference" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,10 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +32,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="3">
@@ -76,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,12 +84,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,17 +455,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -495,22 +492,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Assigned To</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Allocation %</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Coordinators</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Cost</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Coordinators needed</t>
         </is>
       </c>
     </row>
@@ -531,20 +533,21 @@
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
-      </c>
-      <c r="F2" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>2000</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I2" s="5" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -567,20 +570,19 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Kim, Lee</t>
         </is>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>30000</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I3" s="5" t="n">
+        <v>30000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -603,20 +605,19 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Ortiz</t>
         </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>6000</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I4" s="5" t="n">
+        <v>6000</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -639,20 +640,19 @@
           <t>2</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>8000</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I5" s="5" t="n">
+        <v>8000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -675,20 +675,19 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Lee, Ortiz</t>
         </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>12000</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I6" s="5" t="n">
+        <v>12000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -711,20 +710,19 @@
           <t>3</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Kim, Lee</t>
         </is>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>2500</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I7" s="5" t="n">
+        <v>2500</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -747,20 +745,19 @@
           <t>4, 5</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Kim</t>
         </is>
-      </c>
-      <c r="F8" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>3000</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="I8" s="5" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -783,20 +780,19 @@
           <t>6, 7</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Kim, Lee</t>
         </is>
-      </c>
-      <c r="F9" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>4000</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>2</v>
       </c>
+      <c r="I9" s="5" t="n">
+        <v>4000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -819,411 +815,18 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Lee, Ortiz</t>
         </is>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>2500</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>2</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Import this tab. Predecessors are Smartsheet row numbers (A = row 1). Assigned To holds the early-start assignment of three coordinators; Allocation % is 100 per person.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Column or field</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Where</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Smartsheet formula</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Cost per day</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C2" s="6">
-        <f>Cost@row / NETWORKDAYS([Start Date]@row, [End Date]@row)</f>
-        <v/>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Direct cost spread evenly over the activity's workdays</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Workday start</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C3" s="6">
-        <f>NETWORKDAYS([Start Date]$1, [Start Date]@row) - 1</f>
-        <v/>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>0 = project start; matches the notes' day numbers</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Workday finish</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C4" s="6">
-        <f>NETWORKDAYS([Start Date]$1, [End Date]@row)</f>
-        <v/>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Finish day as the notes count it</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Wk 1 PV</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C5" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 2), [Start Date]@row, DATE(2026, 11, 2)), IF([End Date]@row &lt; DATE(2026, 11, 6), [End Date]@row, DATE(2026, 11, 6)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 1: Mon 2 Nov to Fri 6 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Wk 2 PV</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C6" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 9), [Start Date]@row, DATE(2026, 11, 9)), IF([End Date]@row &lt; DATE(2026, 11, 13), [End Date]@row, DATE(2026, 11, 13)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 2: Mon 9 Nov to Fri 13 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Wk 3 PV</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C7" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 16), [Start Date]@row, DATE(2026, 11, 16)), IF([End Date]@row &lt; DATE(2026, 11, 20), [End Date]@row, DATE(2026, 11, 20)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 3: Mon 16 Nov to Fri 20 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Wk 4 PV</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C8" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 23), [Start Date]@row, DATE(2026, 11, 23)), IF([End Date]@row &lt; DATE(2026, 11, 27), [End Date]@row, DATE(2026, 11, 27)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 4: Mon 23 Nov to Fri 27 Nov</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Wk 5 PV</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C9" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 11, 30), [Start Date]@row, DATE(2026, 11, 30)), IF([End Date]@row &lt; DATE(2026, 12, 4), [End Date]@row, DATE(2026, 12, 4)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 5: Mon 30 Nov to Fri 4 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Wk 6 PV</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C10" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 12, 7), [Start Date]@row, DATE(2026, 12, 7)), IF([End Date]@row &lt; DATE(2026, 12, 11), [End Date]@row, DATE(2026, 12, 11)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 6: Mon 7 Dec to Fri 11 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Wk 7 PV</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C11" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 12, 14), [Start Date]@row, DATE(2026, 12, 14)), IF([End Date]@row &lt; DATE(2026, 12, 18), [End Date]@row, DATE(2026, 12, 18)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 7: Mon 14 Dec to Fri 18 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Wk 8 PV</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>column</t>
-        </is>
-      </c>
-      <c r="C12" s="6">
-        <f>MAX(0, NETWORKDAYS(IF([Start Date]@row &gt; DATE(2026, 12, 21), [Start Date]@row, DATE(2026, 12, 21)), IF([End Date]@row &lt; DATE(2026, 12, 25), [End Date]@row, DATE(2026, 12, 25)))) * [Cost per day]@row</f>
-        <v/>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Planned value in week 8: Mon 21 Dec to Fri 25 Dec</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Project finish</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C13" s="6">
-        <f>MAX([End Date]:[End Date])</f>
-        <v/>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Date type</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Workdays</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C14" s="6">
-        <f>MAX([Workday finish]:[Workday finish])</f>
-        <v/>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>25 on the early-start schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Wk n total</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C15" s="6">
-        <f>SUM([Wk 1 PV]:[Wk 1 PV])  (one field per week)</f>
-        <v/>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Weekly planned value</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Cumulative to wk n</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C16" s="6">
-        <f>[Wk 1 total]# + [Wk 2 total]#  (extend per week)</f>
-        <v/>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>The baseline curve</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Total cost</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Sheet Summary</t>
-        </is>
-      </c>
-      <c r="C17" s="6">
-        <f>SUM(Cost:Cost)</f>
-        <v/>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Must read $70,000 under every schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Smartsheet imports values, not formulas. Type each formula once in row 1, then right-click → Convert to Column Formula. Summary fields are typed in the Sheet Summary panel.</t>
-        </is>
+      <c r="I10" s="5" t="n">
+        <v>2500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>